<commit_message>
Add full funnel sheet: marketing -> sales -> retention
Лист «Воронка полная»: А1-А4 маркетинг (показ-клик-лид-квал),
Б1-Б7 продажи по этапам CRM МИГ (касание ≤1ч, событие, собеседование,
оплата, договор, старт), В1-В5 LTV (удержание, апгрейд до 23.11,
кросс-селл, кейсы, рефералка). План-конверсии из факта 2025,
планы для теста 1000 EUR и полного бюджета, узкое место Б2 отмечено

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WaZo4XqSL8CLQw3gc5JhDV
</commit_message>
<xml_diff>
--- a/docs/clients/slozhny-sluchay-tablitsa.xlsx
+++ b/docs/clients/slozhny-sluchay-tablitsa.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet name="Было — Стало" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Тест 1000 €" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Meta ретаргетинг" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Meta холодный" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="VK Реклама" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Посевы Telegram" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Яндекс бренд" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Воронка полная" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Meta ретаргетинг" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Meta холодный" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="VK Реклама" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Посевы Telegram" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Яндекс бренд" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,6 +92,11 @@
       <color rgb="00EDE6DB"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -151,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -211,6 +217,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -761,7 +768,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
@@ -1247,447 +1253,984 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>«Сложный случай» · тест: Meta ретаргетинг</t>
+          <t>«Сложный случай» · полная воронка: маркетинг → продажи → удержание</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>Бюджет теста: 150 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>План-конверсии: факт МИГ 2025 (138 лидов → 10 студентов с рекламы, 7–9%) + бенчмарки. Обновляются фактом еженедельно.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
-        <is>
-          <t>Параметры</t>
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>А. ВОРОНКА МАРКЕТИНГА-РЕКЛАМЫ (бюджет → квал-лид)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Аудитории</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>Посетители mig.institute 90 дн (пиксель стоит) · вовлечённые IG/FB · база лидов 2025–2026 (custom audience по email/телефонам)</t>
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Этап</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Критерий перехода дальше</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Инструмент / канал</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Ответственный</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Метрика этапа</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>План-конверсия</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>Тест 1 000 €</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>Полный 2 500 €</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>Факт</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Гео</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Все страны кроме РФ (Meta в РФ не показывается)</t>
-        </is>
-      </c>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Показ рекламы</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Увидел объявление/пост</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Meta (ретаргетинг+холод), VK, посевы TG, Яндекс бренд, органика IG/TG</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>Таргетолог / агентство</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>Показы, CPM</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>CTR ~1,3% (факт 2026)</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>~150 000</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>~380 000</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Посадочная</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Лендинг «Сложный случай» (после публикации) / регистрация на демо-день</t>
-        </is>
-      </c>
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Клик / переход</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Перешёл на посадочную</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>Лендинг «Сложный случай» / лид-форма / пост</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Таргетолог</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Клики, CPC ~0,4–0,7 €</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>~35% в лид*</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>~2 000</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>~5 000</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Оффер</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>Демо-день + ранняя цена до 30.09</t>
-        </is>
-      </c>
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Лид (заявка/регистрация)</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Оставил контакт: демо-день, 9 лекций, вопрос</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Форма лендинга, лид-форма с квал-вопросами, @iigestalt, WhatsApp</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Формы → единая таблица</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>Лиды, CPL (цель 8–25 € по каналу)</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>~70% квал</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>~80 платн. + ~40 орг. = 120</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>~175 платн. + ~60 орг. = 235</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Креативы</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>S1 «Обещание», S2 «Боль» из ТЗ v2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>KPI и стоп-лосс</t>
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Квал-лид</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Практикующий/студент послед. года; корректные контакты; ответил</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Квал-вопросы формы + первое касание ≤ 1 часа</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер МИГ (контроль — агентство)</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Квал-лиды, цена квал-лида (цель ≤ 20–45 €)</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>→ в воронку продаж</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>~84</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>~165</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>* лид-формы конвертят выше (нет перехода), лендинг ниже, но чище — считаем смешанно; уточняется тестом</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>Цель CPL</t>
-        </is>
-      </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>≤ 10 € (тёплая аудитория)</t>
-        </is>
-      </c>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Б. ВОРОНКА ПРОДАЖ (CRM МИГ: квал-лид → студент)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>Цель квал-CPL</t>
-        </is>
-      </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>≤ 20 €</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Этап</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Критерий перехода дальше</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Инструмент / канал</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Ответственный</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Метрика этапа</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>План-конверсия</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Тест 1 000 €</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Полный 2 500 €</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Факт</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>Стоп-лосс</t>
-        </is>
-      </c>
-      <c r="B14" s="21" t="inlineStr">
-        <is>
-          <t>150 € без квал-лида — стоп и разбор</t>
-        </is>
-      </c>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Б1</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Новый лид в CRM</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Занесён с источником (UTM) и статусом</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>CRM/единая таблица лидов</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер МИГ</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Скорость занесения (день в день)</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Ожидание теста</t>
-        </is>
-      </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <t>~15 лидов, 1–2 продажи</t>
-        </is>
-      </c>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Б2</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Первое касание</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Исходящее в WhatsApp/TG ≤ 1 часа; ответил на сообщение</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>WhatsApp-скрипт (вычитан журналистом)</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер МИГ</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Доля касаний ≤ 1 ч; доля ответов (цель ≥ 50%, факт 2026 — 10%!)</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>~60% в событие</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>~100</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Б3</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Бесплатное событие</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Пришёл на демо-день / MIG.TALKS / посмотрел лекции</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Демо-день, MIG.TALKS, «9 лекций» (автовыдача)</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Агентство (трафик) + МИГ (событие)</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Доходимость (цель ≥ 40–50%, по 2025 — механика работала)</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>~50% в собеседование</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>~25</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Недельный трекинг (заполнять факт; расчётные колонки считаются сами)</t>
-        </is>
-      </c>
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Б4</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Собеседование</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Записался и пришёл на разговор о программе</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Календарь менеджера; приглашение на событии</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер / ведущие</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Доля дошедших до собеседования</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>~45% в оплату</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>~24</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
-        <is>
-          <t>Неделя</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="inlineStr">
-        <is>
-          <t>Расход €</t>
-        </is>
-      </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>Показы</t>
-        </is>
-      </c>
-      <c r="D18" s="23" t="inlineStr">
-        <is>
-          <t>Клики</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>CPC €</t>
-        </is>
-      </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>CTR %</t>
-        </is>
-      </c>
-      <c r="G18" s="23" t="inlineStr">
-        <is>
-          <t>Лиды</t>
-        </is>
-      </c>
-      <c r="H18" s="23" t="inlineStr">
-        <is>
-          <t>CPL €</t>
-        </is>
-      </c>
-      <c r="I18" s="23" t="inlineStr">
-        <is>
-          <t>Квал лиды</t>
-        </is>
-      </c>
-      <c r="J18" s="23" t="inlineStr">
-        <is>
-          <t>Цена квал-лида €</t>
-        </is>
-      </c>
-      <c r="K18" s="23" t="inlineStr">
-        <is>
-          <t>Продажи</t>
-        </is>
-      </c>
-      <c r="L18" s="23" t="inlineStr">
-        <is>
-          <t>CAC €</t>
-        </is>
-      </c>
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Б5</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Оплата (предоплата)</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Внёс предоплату (цикл: медиана ~22 дня с касаниями, до 64 без)</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Оплата ₽ (ИП) / € (Черногория); ранняя цена до 30.09 — ускоритель</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Продажи, CAC (цель ≤ 650 €, факт 2025 — 72 €)</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>~95% договор</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>~6–8</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>~13–17</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>01.09–07.09</t>
-        </is>
-      </c>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24">
-        <f>IFERROR(B19/D19,"")</f>
-        <v/>
-      </c>
-      <c r="F19" s="24">
-        <f>IFERROR(D19/C19*100,"")</f>
-        <v/>
-      </c>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24">
-        <f>IFERROR(B19/G19,"")</f>
-        <v/>
-      </c>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="24">
-        <f>IFERROR(B19/I19,"")</f>
-        <v/>
-      </c>
-      <c r="K19" s="24" t="n"/>
-      <c r="L19" s="24">
-        <f>IFERROR(B19/K19,"")</f>
-        <v/>
-      </c>
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Б6</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Договор</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Подписан договор</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Документы МИГ</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Администратор</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Доля подписанных</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>~100%</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>6–8</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>13–17</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>08.09–14.09</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24">
-        <f>IFERROR(B20/D20,"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="24">
-        <f>IFERROR(D20/C20*100,"")</f>
-        <v/>
-      </c>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24">
-        <f>IFERROR(B20/G20,"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24">
-        <f>IFERROR(B20/I20,"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="24" t="n"/>
-      <c r="L20" s="24">
-        <f>IFERROR(B20/K20,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>15.09–21.09</t>
-        </is>
-      </c>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24">
-        <f>IFERROR(B21/D21,"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="24">
-        <f>IFERROR(D21/C21*100,"")</f>
-        <v/>
-      </c>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24">
-        <f>IFERROR(B21/G21,"")</f>
-        <v/>
-      </c>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="24">
-        <f>IFERROR(B21/I21,"")</f>
-        <v/>
-      </c>
-      <c r="K21" s="24" t="n"/>
-      <c r="L21" s="24">
-        <f>IFERROR(B21/K21,"")</f>
-        <v/>
-      </c>
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Б7</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Начало учёбы</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Вышел на первый модуль (октябрь)</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Онбординг: письмо + чат потока</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>МИГ</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Доля вышедших; NPS первого модуля</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>→ удержание</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>6–8</t>
+        </is>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>13–17</t>
+        </is>
+      </c>
+      <c r="J20" s="16" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
-        <is>
-          <t>22.09–30.09</t>
-        </is>
-      </c>
-      <c r="B22" s="24" t="n"/>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24">
-        <f>IFERROR(B22/D22,"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="24">
-        <f>IFERROR(D22/C22*100,"")</f>
-        <v/>
-      </c>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="24">
-        <f>IFERROR(B22/G22,"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="24" t="n"/>
-      <c r="J22" s="24">
-        <f>IFERROR(B22/I22,"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="24" t="n"/>
-      <c r="L22" s="24">
-        <f>IFERROR(B22/K22,"")</f>
-        <v/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>В. ПОСЛЕ ПРОДАЖИ (LTV: удержание → апгрейд → рефералка)</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
-        </is>
-      </c>
-      <c r="B23" s="25">
-        <f>SUM(B19:B22)</f>
-        <v/>
-      </c>
-      <c r="C23" s="25">
-        <f>SUM(C19:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="25">
-        <f>SUM(D19:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="25">
-        <f>IFERROR(B23/D23,"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="25">
-        <f>IFERROR(D23/C23*100,"")</f>
-        <v/>
-      </c>
-      <c r="G23" s="25">
-        <f>SUM(G19:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="25">
-        <f>IFERROR(B23/G23,"")</f>
-        <v/>
-      </c>
-      <c r="I23" s="25">
-        <f>SUM(I19:I22)</f>
-        <v/>
-      </c>
-      <c r="J23" s="25">
-        <f>IFERROR(B23/I23,"")</f>
-        <v/>
-      </c>
-      <c r="K23" s="25">
-        <f>SUM(K19:K22)</f>
-        <v/>
-      </c>
-      <c r="L23" s="25">
-        <f>IFERROR(B23/K23,"")</f>
-        <v/>
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Этап</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Критерий перехода дальше</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>Инструмент / канал</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Ответственный</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>Метрика этапа</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>План-конверсия</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>Тест 1 000 €</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>Полный 2 500 €</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>Факт</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>В1</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Удержание</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Проходит модули, не отваливается</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Кураторы, супервизии, чат</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>МИГ</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>Посещаемость модулей</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr"/>
+      <c r="I24" s="16" t="inlineStr"/>
+      <c r="J24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>В2</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Апгрейд тарифа</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Повышение тарифа (возможно до 4-й встречи, 23.11)</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Предложение после 2–3 модуля</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Доля апгрейдов, доп. выручка</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>1–2</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>2–4</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>В3</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Кросс-селл</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Конференция случаев (−50%), «Цифра», спецкурсы</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Email/чат потока</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Менеджер</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>Доп. продажи на студента</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr"/>
+      <c r="I26" s="16" t="inlineStr"/>
+      <c r="J26" s="16" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>В4</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Выпуск и кейс</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Закончил программу; согласие на историю</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Кейс-истории (только реальные, с согласия)</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Агентство + МИГ</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>Собранные кейсы</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr"/>
+      <c r="I27" s="16" t="inlineStr"/>
+      <c r="J27" s="16" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>В5</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Рекомендация</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Привёл коллегу (промокод)</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Реферальная программа (механика — в разработке)</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>Агентство + МИГ</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>Рефералы, CAC ~250 € фикс.</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr"/>
+      <c r="I28" s="16" t="inlineStr"/>
+      <c r="J28" s="16" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Сквозные правила: (1) каждый лид имеет источник (UTM) и статус в единой таблице — иначе воронка не считается;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>(2) узкое место сейчас — этап Б2 (в 2026 отвечают ~10% при цели 50%): скорость касания и скрипты чинятся до масштабирования бюджета;</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>(3) еженедельно: факт-колонка заполняется, конверсии пересчитываются, деньги перекладываются в канал-лидер по CAC;</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>(4) числа «Тест/Полный» — план на основе факта 2025 и бенчмарков; это ориентиры, не обещания.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B5:H5"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1718,14 +2261,14 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>«Сложный случай» · тест: Meta холодный</t>
+          <t>«Сложный случай» · тест: Meta ретаргетинг</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Бюджет теста: 250 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
+          <t>Бюджет теста: 150 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
         </is>
       </c>
     </row>
@@ -1744,7 +2287,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Интересы: Psychology, Psychotherapy, Gestalt therapy · язык русский · 27–55</t>
+          <t>Посетители mig.institute 90 дн (пиксель стоит) · вовлечённые IG/FB · база лидов 2025–2026 (custom audience по email/телефонам)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +2299,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Группа 1: Германия+Израиль · Группа 2: Сербия/Черногория/Хорватия</t>
+          <t>Все страны кроме РФ (Meta в РФ не показывается)</t>
         </is>
       </c>
     </row>
@@ -1768,7 +2311,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Лендинг «Сложный случай» / демо-день; параллельно лидформа с квал-вопросами (тест качества)</t>
+          <t>Лендинг «Сложный случай» (после публикации) / регистрация на демо-день</t>
         </is>
       </c>
     </row>
@@ -1792,7 +2335,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>S1–S4 из ТЗ v2; скрининг по CTR (мин. 500 показов на вариант до выводов)</t>
+          <t>S1 «Обещание», S2 «Боль» из ТЗ v2</t>
         </is>
       </c>
     </row>
@@ -1811,15 +2354,9 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>≤ 25 €</t>
-        </is>
-      </c>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
+          <t>≤ 10 € (тёплая аудитория)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
@@ -1829,15 +2366,9 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>≤ 45 €</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
+          <t>≤ 20 €</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
@@ -1847,15 +2378,9 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Объявление: CPL&gt;40 € при 500+ показов — выкл. Канал: 250 € без квал-лида — стоп</t>
-        </is>
-      </c>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
+          <t>150 € без квал-лида — стоп и разбор</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
@@ -1865,15 +2390,9 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>~10 лидов, ~1 продажа</t>
-        </is>
-      </c>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
+          <t>~15 лидов, 1–2 продажи</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -2169,14 +2688,14 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>«Сложный случай» · тест: VK Реклама</t>
+          <t>«Сложный случай» · тест: Meta холодный</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Бюджет теста: 200 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
+          <t>Бюджет теста: 250 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2714,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Слой 1 (тёплый): подписчики сообщества VK МИГ · Слой 2: интересы психология + активные в сообществах конкурентов (МИГиП, МГИ)</t>
+          <t>Интересы: Psychology, Psychotherapy, Gestalt therapy · язык русский · 27–55</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2726,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>РФ (кабинет на ИП, оплата в ₽)</t>
+          <t>Группа 1: Германия+Израиль · Группа 2: Сербия/Черногория/Хорватия</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2738,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Лендинг / лид-форма VK с квал-вопросами (A/B)</t>
+          <t>Лендинг «Сложный случай» / демо-день; параллельно лидформа с квал-вопросами (тест качества)</t>
         </is>
       </c>
     </row>
@@ -2231,19 +2750,19 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Демо-день + ранняя цена до 30.09; цены в рублях</t>
+          <t>Демо-день + ранняя цена до 30.09</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>Маркировка</t>
+          <t>Креативы</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Автоматическая (erid), данные рекламодателя — ИП</t>
+          <t>S1–S4 из ТЗ v2; скрининг по CTR (мин. 500 показов на вариант до выводов)</t>
         </is>
       </c>
     </row>
@@ -2262,15 +2781,9 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>≤ 8 € (≈800 ₽)</t>
-        </is>
-      </c>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
+          <t>≤ 25 €</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
@@ -2280,15 +2793,9 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>≤ 18 €</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
+          <t>≤ 45 €</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
@@ -2298,15 +2805,9 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>120 € без квал-лида — пауза, смена слоя аудитории</t>
-        </is>
-      </c>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
+          <t>Объявление: CPL&gt;40 € при 500+ показов — выкл. Канал: 250 € без квал-лида — стоп</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
@@ -2316,15 +2817,9 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>~25 лидов, 1–2 продажи</t>
-        </is>
-      </c>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
+          <t>~10 лидов, ~1 продажа</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -2595,295 +3090,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>«Сложный случай» · тест: посевы в Telegram-каналах</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>Бюджет теста: 300 €  ·  4–6 каналов  ·  окно: 01–30.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="17" t="inlineStr">
-        <is>
-          <t>Отбор каналов</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>Психологические профессиональные каналы; проверка через TGStat: динамика подписчиков, ER, просмотры/пост (протокол R06). Покупка только после проверки</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Формат</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>Нативный пост-разбор («как психологу работать со сложным случаем») + анонс демо-дня; согласование текста с автором канала</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Маркировка</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>РФ-аудитория: erid через ОРД от ИП — обязательно в каждом посте</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Цена перехода ≤ 1,5 € · CPL ≤ 15 € · стоп-лосс: после первых 2 каналов сверка, дальше только аналоги лучших</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Канал</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Дата поста</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Цена €</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Подписчиков</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Охват поста</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>Переходы</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>Цена перехода €</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Лиды</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>CPL €</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="inlineStr">
-        <is>
-          <t>Продажи</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="26" t="n"/>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="26" t="n"/>
-      <c r="F10" s="26" t="n"/>
-      <c r="G10" s="24">
-        <f>IFERROR(C10/F10,"")</f>
-        <v/>
-      </c>
-      <c r="H10" s="26" t="n"/>
-      <c r="I10" s="24">
-        <f>IFERROR(C10/H10,"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="26" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="26" t="n"/>
-      <c r="B11" s="26" t="n"/>
-      <c r="C11" s="26" t="n"/>
-      <c r="D11" s="26" t="n"/>
-      <c r="E11" s="26" t="n"/>
-      <c r="F11" s="26" t="n"/>
-      <c r="G11" s="24">
-        <f>IFERROR(C11/F11,"")</f>
-        <v/>
-      </c>
-      <c r="H11" s="26" t="n"/>
-      <c r="I11" s="24">
-        <f>IFERROR(C11/H11,"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="26" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="n"/>
-      <c r="B12" s="26" t="n"/>
-      <c r="C12" s="26" t="n"/>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="26" t="n"/>
-      <c r="F12" s="26" t="n"/>
-      <c r="G12" s="24">
-        <f>IFERROR(C12/F12,"")</f>
-        <v/>
-      </c>
-      <c r="H12" s="26" t="n"/>
-      <c r="I12" s="24">
-        <f>IFERROR(C12/H12,"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="26" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="n"/>
-      <c r="B13" s="26" t="n"/>
-      <c r="C13" s="26" t="n"/>
-      <c r="D13" s="26" t="n"/>
-      <c r="E13" s="26" t="n"/>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="24">
-        <f>IFERROR(C13/F13,"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="26" t="n"/>
-      <c r="I13" s="24">
-        <f>IFERROR(C13/H13,"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="26" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="26" t="n"/>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-      <c r="D14" s="26" t="n"/>
-      <c r="E14" s="26" t="n"/>
-      <c r="F14" s="26" t="n"/>
-      <c r="G14" s="24">
-        <f>IFERROR(C14/F14,"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="26" t="n"/>
-      <c r="I14" s="24">
-        <f>IFERROR(C14/H14,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="26" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="26" t="n"/>
-      <c r="B15" s="26" t="n"/>
-      <c r="C15" s="26" t="n"/>
-      <c r="D15" s="26" t="n"/>
-      <c r="E15" s="26" t="n"/>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="24">
-        <f>IFERROR(C15/F15,"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="26" t="n"/>
-      <c r="I15" s="24">
-        <f>IFERROR(C15/H15,"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="26" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
-        </is>
-      </c>
-      <c r="C16" s="17">
-        <f>SUM(C10:C15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="17">
-        <f>SUM(E10:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="17">
-        <f>SUM(F10:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="17">
-        <f>IFERROR(C16/F16,"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="17">
-        <f>SUM(H10:H15)</f>
-        <v/>
-      </c>
-      <c r="I16" s="17">
-        <f>IFERROR(C16/H16,"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="17">
-        <f>SUM(J10:J15)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B4:I4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2909,14 +3115,14 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>«Сложный случай» · тест: Яндекс бренд</t>
+          <t>«Сложный случай» · тест: VK Реклама</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Бюджет теста: 100 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
+          <t>Бюджет теста: 200 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
         </is>
       </c>
     </row>
@@ -2930,60 +3136,60 @@
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Аудитории</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Поисковая бренд-защита (только брендовые запросы)</t>
+          <t>Слой 1 (тёплый): подписчики сообщества VK МИГ · Слой 2: интересы психология + активные в сообществах конкурентов (МИГиП, МГИ)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Семантика</t>
+          <t>Гео</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>«миг институт гештальта», «международный институт гештальта», варианты написания; минус-слова от МИГиП/МГИ курсов</t>
+          <t>РФ (кабинет на ИП, оплата в ₽)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Гео</t>
+          <t>Посадочная</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>РФ + СНГ</t>
+          <t>Лендинг / лид-форма VK с квал-вопросами (A/B)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Посадочная</t>
+          <t>Оффер</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>mig.institute (или лендинг «Сложного случая» для запросов с «ппк/повышение квалификации»)</t>
+          <t>Демо-день + ранняя цена до 30.09; цены в рублях</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>Задача</t>
+          <t>Маркировка</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Не отдавать готовых покупателей конкурентам-однофамильцам; проверить, кто рекламируется по бренду МИГ</t>
+          <t>Автоматическая (erid), данные рекламодателя — ИП</t>
         </is>
       </c>
     </row>
@@ -2997,38 +3203,26 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>Цель CPC</t>
+          <t>Цель CPL</t>
         </is>
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>≤ 0,3 € (брендовые клики дёшевы)</t>
-        </is>
-      </c>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
+          <t>≤ 8 € (≈800 ₽)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>Цель CPL</t>
+          <t>Цель квал-CPL</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>≤ 10 €</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
+          <t>≤ 18 €</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
@@ -3038,15 +3232,9 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Не расширять на небрендовые запросы в рамках теста</t>
-        </is>
-      </c>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
+          <t>120 € без квал-лида — пауза, смена слоя аудитории</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
@@ -3056,15 +3244,725 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
+          <t>~25 лидов, 1–2 продажи</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Недельный трекинг (заполнять факт; расчётные колонки считаются сами)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>Неделя</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Расход €</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Показы</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Клики</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>CPC €</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>CTR %</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>Лиды</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>CPL €</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>Квал лиды</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>Цена квал-лида €</t>
+        </is>
+      </c>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>Продажи</t>
+        </is>
+      </c>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>CAC €</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>01.09–07.09</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24">
+        <f>IFERROR(B19/D19,"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="24">
+        <f>IFERROR(D19/C19*100,"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="24" t="n"/>
+      <c r="H19" s="24">
+        <f>IFERROR(B19/G19,"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="24" t="n"/>
+      <c r="J19" s="24">
+        <f>IFERROR(B19/I19,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="24" t="n"/>
+      <c r="L19" s="24">
+        <f>IFERROR(B19/K19,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>08.09–14.09</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24">
+        <f>IFERROR(B20/D20,"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="24">
+        <f>IFERROR(D20/C20*100,"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="24" t="n"/>
+      <c r="H20" s="24">
+        <f>IFERROR(B20/G20,"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="24" t="n"/>
+      <c r="J20" s="24">
+        <f>IFERROR(B20/I20,"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="24" t="n"/>
+      <c r="L20" s="24">
+        <f>IFERROR(B20/K20,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>15.09–21.09</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24">
+        <f>IFERROR(B21/D21,"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="24">
+        <f>IFERROR(D21/C21*100,"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="24" t="n"/>
+      <c r="H21" s="24">
+        <f>IFERROR(B21/G21,"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="24" t="n"/>
+      <c r="J21" s="24">
+        <f>IFERROR(B21/I21,"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="24" t="n"/>
+      <c r="L21" s="24">
+        <f>IFERROR(B21/K21,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>22.09–30.09</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24">
+        <f>IFERROR(B22/D22,"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="24">
+        <f>IFERROR(D22/C22*100,"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="24" t="n"/>
+      <c r="H22" s="24">
+        <f>IFERROR(B22/G22,"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="24" t="n"/>
+      <c r="J22" s="24">
+        <f>IFERROR(B22/I22,"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="24" t="n"/>
+      <c r="L22" s="24">
+        <f>IFERROR(B22/K22,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B23" s="25">
+        <f>SUM(B19:B22)</f>
+        <v/>
+      </c>
+      <c r="C23" s="25">
+        <f>SUM(C19:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="25">
+        <f>SUM(D19:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="25">
+        <f>IFERROR(B23/D23,"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="25">
+        <f>IFERROR(D23/C23*100,"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="25">
+        <f>SUM(G19:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="25">
+        <f>IFERROR(B23/G23,"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="25">
+        <f>SUM(I19:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="25">
+        <f>IFERROR(B23/I23,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="25">
+        <f>SUM(K19:K22)</f>
+        <v/>
+      </c>
+      <c r="L23" s="25">
+        <f>IFERROR(B23/K23,"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B5:H5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>«Сложный случай» · тест: посевы в Telegram-каналах</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Бюджет теста: 300 €  ·  4–6 каналов  ·  окно: 01–30.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Отбор каналов</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Психологические профессиональные каналы; проверка через TGStat: динамика подписчиков, ER, просмотры/пост (протокол R06). Покупка только после проверки</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Формат</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Нативный пост-разбор («как психологу работать со сложным случаем») + анонс демо-дня; согласование текста с автором канала</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Маркировка</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>РФ-аудитория: erid через ОРД от ИП — обязательно в каждом посте</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Цена перехода ≤ 1,5 € · CPL ≤ 15 € · стоп-лосс: после первых 2 каналов сверка, дальше только аналоги лучших</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Канал</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Дата поста</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Цена €</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Подписчиков</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Охват поста</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Переходы</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>Цена перехода €</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>Лиды</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>CPL €</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>Продажи</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="n"/>
+      <c r="B10" s="26" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="26" t="n"/>
+      <c r="G10" s="24">
+        <f>IFERROR(C10/F10,"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="26" t="n"/>
+      <c r="I10" s="24">
+        <f>IFERROR(C10/H10,"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="26" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="n"/>
+      <c r="B11" s="26" t="n"/>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="26" t="n"/>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="24">
+        <f>IFERROR(C11/F11,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="26" t="n"/>
+      <c r="I11" s="24">
+        <f>IFERROR(C11/H11,"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="26" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="n"/>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="26" t="n"/>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="24">
+        <f>IFERROR(C12/F12,"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="26" t="n"/>
+      <c r="I12" s="24">
+        <f>IFERROR(C12/H12,"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="26" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="n"/>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="24">
+        <f>IFERROR(C13/F13,"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="26" t="n"/>
+      <c r="I13" s="24">
+        <f>IFERROR(C13/H13,"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="26" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="26" t="n"/>
+      <c r="F14" s="26" t="n"/>
+      <c r="G14" s="24">
+        <f>IFERROR(C14/F14,"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="26" t="n"/>
+      <c r="I14" s="24">
+        <f>IFERROR(C14/H14,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="26" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="n"/>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+      <c r="D15" s="26" t="n"/>
+      <c r="E15" s="26" t="n"/>
+      <c r="F15" s="26" t="n"/>
+      <c r="G15" s="24">
+        <f>IFERROR(C15/F15,"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="26" t="n"/>
+      <c r="I15" s="24">
+        <f>IFERROR(C15/H15,"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="26" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="C16" s="17">
+        <f>SUM(C10:C15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>SUM(E10:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="17">
+        <f>SUM(F10:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="17">
+        <f>IFERROR(C16/F16,"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="17">
+        <f>SUM(H10:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>IFERROR(C16/H16,"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="17">
+        <f>SUM(J10:J15)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B4:I4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>«Сложный случай» · тест: Яндекс бренд</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Бюджет теста: 100 €  ·  окно: 01–30.09 (ранняя цена до 30.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Параметры</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Поисковая бренд-защита (только брендовые запросы)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Семантика</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>«миг институт гештальта», «международный институт гештальта», варианты написания; минус-слова от МИГиП/МГИ курсов</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Гео</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>РФ + СНГ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Посадочная</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>mig.institute (или лендинг «Сложного случая» для запросов с «ппк/повышение квалификации»)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Задача</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Не отдавать готовых покупателей конкурентам-однофамильцам; проверить, кто рекламируется по бренду МИГ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>KPI и стоп-лосс</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Цель CPC</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>≤ 0,3 € (брендовые клики дёшевы)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>Цель CPL</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>≤ 10 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>Стоп-лосс</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Не расширять на небрендовые запросы в рамках теста</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Ожидание теста</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
           <t>~10 лидов высочайшего качества</t>
         </is>
       </c>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Update funnel owners: Tina K. for marketing, ROP Valya + 2 managers for sales
Убран «агентство» из ответственных; команда зафиксирована в досье:
Тина К. - исследования/редизайн/маркетинг/реклама; РОП Валя + 2
менеджера - все этапы продаж

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WaZo4XqSL8CLQw3gc5JhDV
</commit_message>
<xml_diff>
--- a/docs/clients/slozhny-sluchay-tablitsa.xlsx
+++ b/docs/clients/slozhny-sluchay-tablitsa.xlsx
@@ -1282,6 +1282,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -1364,7 +1365,7 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Таргетолог / агентство</t>
+          <t>Тина К.</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
@@ -1412,7 +1413,7 @@
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Таргетолог</t>
+          <t>Тина К.</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -1460,7 +1461,7 @@
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Формы → единая таблица</t>
+          <t>Тина К. (настройка форм)</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
@@ -1508,7 +1509,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>Менеджер МИГ (контроль — агентство)</t>
+          <t>Менеджеры Вали (2)</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
@@ -1540,6 +1541,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
@@ -1622,7 +1624,7 @@
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>Менеджер МИГ</t>
+          <t>Менеджеры Вали (2)</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
@@ -1670,7 +1672,7 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>Менеджер МИГ</t>
+          <t>Менеджеры Вали (2)</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
@@ -1718,7 +1720,7 @@
       </c>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>Агентство (трафик) + МИГ (событие)</t>
+          <t>Тина К. (трафик) + МИГ (событие)</t>
         </is>
       </c>
       <c r="F16" s="16" t="inlineStr">
@@ -1766,7 +1768,7 @@
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>Менеджер / ведущие</t>
+          <t>Менеджеры Вали / ведущие</t>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -1814,7 +1816,7 @@
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>Менеджер</t>
+          <t>РОП Валя</t>
         </is>
       </c>
       <c r="F18" s="16" t="inlineStr">
@@ -1935,6 +1937,7 @@
       </c>
       <c r="J20" s="16" t="inlineStr"/>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -2057,7 +2060,7 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>Менеджер</t>
+          <t>РОП Валя</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
@@ -2105,7 +2108,7 @@
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>Менеджер</t>
+          <t>РОП Валя</t>
         </is>
       </c>
       <c r="F26" s="16" t="inlineStr">
@@ -2145,7 +2148,7 @@
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>Агентство + МИГ</t>
+          <t>Тина К. + МИГ</t>
         </is>
       </c>
       <c r="F27" s="16" t="inlineStr">
@@ -2185,7 +2188,7 @@
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>Агентство + МИГ</t>
+          <t>Тина К. + РОП Валя</t>
         </is>
       </c>
       <c r="F28" s="16" t="inlineStr">
@@ -2202,6 +2205,7 @@
       <c r="I28" s="16" t="inlineStr"/>
       <c r="J28" s="16" t="inlineStr"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>

</xml_diff>